<commit_message>
Added RDF data schemes and fixed visual schemes for health-table01-05
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/health-table01.xlsx
+++ b/sources/table_normalization/xlsx/health-table01.xlsx
@@ -137,8 +137,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="2">
-    <numFmt numFmtId="166" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="168" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -220,19 +220,20 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -1459,12 +1460,12 @@
     <row r="3" spans="1:4"/>
     <row r="4" spans="1:4"/>
     <row r="5" spans="1:4" ht="18.5">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
     </row>
     <row r="6" spans="1:4" ht="15.5">
       <c r="A6" s="1" t="s">
@@ -1476,16 +1477,16 @@
       </c>
     </row>
     <row r="7" spans="1:4">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1561,12 +1562,12 @@
     </row>
     <row r="13" spans="1:4"/>
     <row r="14" spans="1:4" ht="18.5">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
     </row>
     <row r="15" spans="1:4" ht="15.5">
       <c r="A15" s="1" t="s">
@@ -1578,16 +1579,16 @@
       </c>
     </row>
     <row r="16" spans="1:4">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="D16" s="6" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1662,12 +1663,12 @@
       </c>
     </row>
     <row r="22" spans="1:4" ht="18.5">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
     </row>
     <row r="23" spans="1:4" ht="15.5">
       <c r="A23" s="1" t="s">
@@ -1679,16 +1680,16 @@
       </c>
     </row>
     <row r="24" spans="1:4">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="D24" s="6" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1764,12 +1765,12 @@
     </row>
     <row r="30" spans="1:4"/>
     <row r="31" spans="1:4" ht="18.5">
-      <c r="A31" s="4" t="s">
+      <c r="A31" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B31" s="4"/>
-      <c r="C31" s="4"/>
-      <c r="D31" s="4"/>
+      <c r="B31" s="5"/>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
     </row>
     <row r="32" spans="1:4" ht="15.5">
       <c r="A32" s="1" t="s">
@@ -1781,16 +1782,16 @@
       </c>
     </row>
     <row r="33" spans="1:4">
-      <c r="A33" s="5" t="s">
+      <c r="A33" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B33" s="5" t="s">
+      <c r="B33" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="C33" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D33" s="5" t="s">
+      <c r="D33" s="6" t="s">
         <v>28</v>
       </c>
     </row>

</xml_diff>